<commit_message>
Documento: inspeção visual mensal (12/ano) e custo da hora do mecânico (Portal Salário/Novo Caged, CBO 9113-05, ref. 15)
- Quadro 2: inspeção visual mensal
- 2.2.4: inspeções visuais mensais de vazamento, ruído e temperatura (o nível é conferido
  no complemento, com bloqueio, como validado com o professor)
- Custo: R$ 3.150/mês, 44 h/semana → R$ 14,32/h (÷ 220 h), sem encargos (conservador)
- Planilha já com 12 intervenções/ano e R$ 14,32/h preenchidos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cronometragem_QRCode.xlsx
+++ b/Cronometragem_QRCode.xlsx
@@ -124,7 +124,7 @@
     <t xml:space="preserve">Custo da hora do mecânico (R$)</t>
   </si>
   <si>
-    <t xml:space="preserve">citar a fonte no documento</t>
+    <t xml:space="preserve">R$ 3.150/mês ÷ 220 h – Portal Salário/Novo Caged, CBO 9113-05</t>
   </si>
   <si>
     <t xml:space="preserve">Tempo ganho por intervenção (s)</t>
@@ -864,7 +864,9 @@
       <c r="A10" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="4"/>
+      <c r="B10" s="4" t="n">
+        <v>14.32</v>
+      </c>
       <c r="C10" s="0" t="s">
         <v>33</v>
       </c>

</xml_diff>